<commit_message>
actulizar tabla del protocolo
</commit_message>
<xml_diff>
--- a/protocolo_pruebas_WIP_v2.xlsx
+++ b/protocolo_pruebas_WIP_v2.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LAC\2026\Sebastian\Tesis_pruebas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44F22DE-5865-4E0E-B1B7-072BFAF895C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D7EBB6-8270-41B0-94F8-702E05C93602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{63CCC3CA-1558-461E-B0B6-AA37C2AD9662}"/>
+    <workbookView xWindow="-110" yWindow="-10910" windowWidth="19420" windowHeight="10300" xr2:uid="{63CCC3CA-1558-461E-B0B6-AA37C2AD9662}"/>
   </bookViews>
   <sheets>
     <sheet name="Fase Simulacion" sheetId="1" r:id="rId1"/>
-    <sheet name="Fase Emulacion" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="100">
   <si>
     <t>Numero de Prueba</t>
   </si>
@@ -184,9 +183,6 @@
   </si>
   <si>
     <t>T5</t>
-  </si>
-  <si>
-    <t>Verificar deteccion de DNS spoofing</t>
   </si>
   <si>
     <t>Víctima -&gt; Atacante (Intercepción DNS) -&gt; IP Atacante (Sitio Falso)</t>
@@ -268,19 +264,6 @@
   </si>
   <si>
     <t>1. La tabla ARP de la Víctima asocia la IP del Gateway con la dirección MAC del Atacante.</t>
-  </si>
-  <si>
-    <t>1. En la Víctima, limpiar caché DNS (ipconfig /flushdns o similar).</t>
-  </si>
-  <si>
-    <t>2. En el Atacante, iniciar el servicio de spoofing DNS (sudo ettercap -G).</t>
-  </si>
-  <si>
-    <t>3. En la Víctima, intentar acceder vía navegador web a nokia.com.</t>
-  </si>
-  <si>
-    <t>1. El comando nslookup devuelve la IP del Atacante para el dominio consultado.
-2. El navegador de la Víctima despliega el contenido alojado en el servidor web del Atacante.</t>
   </si>
   <si>
     <t>DESARROLLO DE UN SISTEMA DE GESTIÓN DE EVENTOS E INFORMACIÓN DE SEGURIDAD, DE BAJO COSTO, BASADO EN SOFTWARE LIBRE, ESPECIALIZADO EN LA DETECCIÓN Y APOYO A LA RESPUESTA ANTE ATAQUES DE TIPO RANSOMWARE.</t>
@@ -311,42 +294,6 @@
     <t>Fecha: Abril del 2026</t>
   </si>
   <si>
-    <t># de prueba</t>
-  </si>
-  <si>
-    <t>Prueba de conectividad completa</t>
-  </si>
-  <si>
-    <t>conexión de todos los nodos</t>
-  </si>
-  <si>
-    <t>En cada máquina de la LAN interna, hacer ping a 10.0.0.1, luego a 192.168.0.10, luego a 1.1.1.1</t>
-  </si>
-  <si>
-    <t>T11</t>
-  </si>
-  <si>
-    <t>T12</t>
-  </si>
-  <si>
-    <t>T13</t>
-  </si>
-  <si>
-    <t>T14</t>
-  </si>
-  <si>
-    <t>T15</t>
-  </si>
-  <si>
-    <t>T16</t>
-  </si>
-  <si>
-    <t>T17</t>
-  </si>
-  <si>
-    <t>T18</t>
-  </si>
-  <si>
     <t>1. Se Habilita ip forwarding en la maquina atacante</t>
   </si>
   <si>
@@ -373,13 +320,49 @@
   <si>
     <t>Retorna la secuencia 
 20:39:25.692987 ARP, reply 10,0,2,15 is -at 08:00:27:8a:35:d2, length 46 ….</t>
+  </si>
+  <si>
+    <t>Verificar deteccion de DNS spoofing	Víctima -&gt; Atacante (Intercepción DNS) -&gt; IP Atacante (Sitio Falso)</t>
+  </si>
+  <si>
+    <t>1.	En el Atacante, iniciar el servicio de spoofing DNS (sudo ettercap -G)</t>
+  </si>
+  <si>
+    <t>2. una vez en la herramienta gráfica, es necesario habilitar el plugin para dns spoofing en el apartado de plugins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.se hace un escaneo de la red, con el botón hosts list y se selecciona el host al que se desea hacer el spoofing </t>
+  </si>
+  <si>
+    <t>4. dentro del menu de mitm, hay que activar la opción de arp spoofing para poner en marcha el ataque</t>
+  </si>
+  <si>
+    <t>5. En la Víctima, intentar acceder vía navegador web a nokia.com.</t>
+  </si>
+  <si>
+    <t>Instalación del componente</t>
+  </si>
+  <si>
+    <t>Salida de los elementos de red definidos en el host</t>
+  </si>
+  <si>
+    <t>El comando nslookup devuelve la IP del Atacante para el dominio consultado.</t>
+  </si>
+  <si>
+    <t>Selección de la opción mitm</t>
+  </si>
+  <si>
+    <t>Activación del servicio</t>
+  </si>
+  <si>
+    <t>Visualización en el navegador de la página intervenida</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -418,21 +401,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -441,19 +411,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="0" tint="-0.14999847407452621"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -482,32 +446,14 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
+      <left style="thin">
         <color indexed="64"/>
-      </top>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -523,12 +469,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -536,77 +508,70 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -991,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88F9D26C-F01D-4F0D-9B0D-9A3523484190}">
-  <dimension ref="B1:I38"/>
+  <dimension ref="B1:I37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.6328125" customWidth="1"/>
@@ -1005,65 +970,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="23" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C1" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="C1" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
     </row>
     <row r="2" spans="2:8" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
+      <c r="C2" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
+      <c r="C3" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
     </row>
     <row r="4" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="8" t="s">
         <v>5</v>
       </c>
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1084,45 +1049,45 @@
       <c r="B8" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-1_W2_ping_gateway.png", "Ver Evidencia PCWin11-1")</f>
         <v>Ver Evidencia PCWin11-1</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="25"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
       <c r="F9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="6" t="str">
+        <v>63</v>
+      </c>
+      <c r="G9" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-1_W2_ping_gateway.png", "Ver Evidencia PCWin11-2")</f>
         <v>Ver Evidencia PCWin11-2</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B10" s="25"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
       <c r="F10" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G10" s="6" t="str">
+        <v>64</v>
+      </c>
+      <c r="G10" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-1_W3_ping_gateway.png", "Ver Evidencia PCWin11-3")</f>
         <v>Ver Evidencia PCWin11-3</v>
       </c>
@@ -1131,45 +1096,45 @@
       <c r="B11" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>72</v>
+      <c r="E11" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="6" t="str">
+        <v>65</v>
+      </c>
+      <c r="G11" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-2_W1_ping_northbound.png", "Ver Evidencia PCWin11-1")</f>
         <v>Ver Evidencia PCWin11-1</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" s="25"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="5"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="16"/>
       <c r="F12" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="G12" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-2_W2_ping_northbound.png", "Ver Evidencia PCWin11-2")</f>
         <v>Ver Evidencia PCWin11-2</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B13" s="25"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="5"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="16"/>
       <c r="F13" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13" s="6" t="str">
+        <v>67</v>
+      </c>
+      <c r="G13" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-2_W3_ping_northbound.png", "Ver Evidencia PCWin11-3")</f>
         <v>Ver Evidencia PCWin11-3</v>
       </c>
@@ -1178,390 +1143,424 @@
       <c r="B14" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>73</v>
+      <c r="E14" s="16" t="s">
+        <v>72</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="6" t="str">
+        <v>68</v>
+      </c>
+      <c r="G14" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-3_W1_ping_nokia.png", "Ver Evidencia PCWin11-1")</f>
         <v>Ver Evidencia PCWin11-1</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B15" s="25"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G15" s="6" t="str">
+        <v>69</v>
+      </c>
+      <c r="G15" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-3_W2_ping_nokia.png", "Ver Evidencia PCWin11-2")</f>
         <v>Ver Evidencia PCWin11-2</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="25"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G16" s="6" t="str">
+        <v>70</v>
+      </c>
+      <c r="G16" s="5" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T1-3_W3_ping_nokia.png", "Ver Evidencia PCWin11-3")</f>
         <v>Ver Evidencia PCWin11-3</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="58" x14ac:dyDescent="0.35">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="8" t="str">
+      <c r="G17" s="6" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T2_docker_ps_galp.png", "Ver Evidencia Stack GLAP")</f>
         <v>Ver Evidencia Stack GLAP</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B18" s="27" t="s">
+    <row r="18" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B18" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G18" s="9" t="str">
+      <c r="G18" s="7" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T2-1_galp_targets_up.png", "Ver Evidencia Verificacion de servicios del stack")</f>
         <v>Ver Evidencia Verificacion de servicios del stack</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="9" t="str">
+      <c r="G19" s="7" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T3_suricata_zeek_docker_ps.png", "Ver Evidencia de activación de Zuticata y Zeek")</f>
         <v>Ver Evidencia de activación de Zuticata y Zeek</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G20" s="9" t="str">
+      <c r="G20" s="7" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T3-1_utmstack_docker_ps.png", "Ver Evidencia de activación UTMStack")</f>
         <v>Ver Evidencia de activación UTMStack</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G21" s="9" t="str">
+      <c r="G21" s="7" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T3-2_wazuh_docker_ps.png", "Ver Evidencia de activación servicios Wazuh")</f>
         <v>Ver Evidencia de activación servicios Wazuh</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="F22" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="G22" s="29"/>
+      <c r="E22" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G22" s="14" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T4_N1_ip_forward.png", "Ver Evidencia habilitacion del forwarding")</f>
+        <v>Ver Evidencia habilitacion del forwarding</v>
+      </c>
     </row>
     <row r="23" spans="2:9" ht="35.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="19"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="G23" s="9" t="str">
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G23" s="15" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T4_arp_initial.png", "Ver Evidencia MAC legitima del Gateway")</f>
         <v>Ver Evidencia MAC legitima del Gateway</v>
       </c>
     </row>
     <row r="24" spans="2:9" ht="46" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="19"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="F24" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="G24" s="21" t="str">
-        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T4_arpspoof_attack.png", "Ver Evidencia envenenamiento (Arpsoof)")</f>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G24" s="15" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T4_N2_Envenenamiento.png", "Ver Evidencia envenenamiento (Arpsoof)")</f>
         <v>Ver Evidencia envenenamiento (Arpsoof)</v>
       </c>
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="2:9" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="20"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="F25" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="G25" s="9" t="str">
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="15" t="str">
         <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T4_arp_after_attack.png", "Ver Evidencia ARP después del ataque")</f>
         <v>Ver Evidencia ARP después del ataque</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="47" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="22"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="F26" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="G26" s="21"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G26" s="15" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T4_N3_TCPDump.png", "Ver Evidencia aplicación del TCPDump")</f>
+        <v>Ver Evidencia aplicación del TCPDump</v>
+      </c>
     </row>
     <row r="27" spans="2:9" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G27" s="7" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T5_ettercap_start.png", "Ver Evidencia iniciación del servicio spoofing")</f>
+        <v>Ver Evidencia iniciación del servicio spoofing</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G28" s="7" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T5_ettercap_dns_plugin.png", "Ver Evidencia habilitación del plugin")</f>
+        <v>Ver Evidencia habilitación del plugin</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G29" s="7" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T5_ettercap_hosts_scan.png", "Ver Evidencia selección del host")</f>
+        <v>Ver Evidencia selección del host</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G30" s="7" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T5_ettercap_arp_spoofing.png", "Ver Evidencia activación ARP Spoofing")</f>
+        <v>Ver Evidencia activación ARP Spoofing</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G31" s="7" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T5_ettercap_attack_active.png", "Ver Evidencia del servicio activado")</f>
+        <v>Ver Evidencia del servicio activado</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G32" s="7" t="str">
+        <f>HYPERLINK("https://github.com/jclavijomartinez/tesis/blob/main/imagenes/T5_victim_fake_site.png", "Ver Evidencia del sitio falso")</f>
+        <v>Ver Evidencia del sitio falso</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="B33" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E27" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="G27" s="7"/>
-    </row>
-    <row r="28" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B28" s="27"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-    </row>
-    <row r="29" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B29" s="27"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B30" s="27"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="C33" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
     </row>
     <row r="34" spans="2:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="B34" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="C34" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
     </row>
     <row r="35" spans="2:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="B35" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C35" s="7" t="s">
+      <c r="B35" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
     </row>
     <row r="36" spans="2:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="B36" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C36" s="7" t="s">
+      <c r="B36" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D36" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-    </row>
-    <row r="37" spans="2:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="B37" s="7" t="s">
+      <c r="C36" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="D36" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B37" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D37" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-    </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B38" s="7" t="s">
+      <c r="C37" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C38" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
+      <c r="D37" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="22">
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="E11:E13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="B11:B13"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="C1:G1"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="B22:B25"/>
     <mergeCell ref="C22:C26"/>
     <mergeCell ref="D22:D26"/>
     <mergeCell ref="C14:C16"/>
     <mergeCell ref="D14:D16"/>
     <mergeCell ref="E14:E16"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="E11:E13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="C27:C32"/>
+    <mergeCell ref="D27:D32"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
@@ -1573,220 +1572,4 @@
   </ignoredErrors>
   <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C15084C-B743-40A5-87FE-3A26809A7529}">
-  <dimension ref="B6:G24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="6" spans="2:7" ht="72" x14ac:dyDescent="0.35">
-      <c r="B6" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" ht="170.5" x14ac:dyDescent="0.35">
-      <c r="B7" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-    </row>
-    <row r="8" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B8" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-    </row>
-    <row r="9" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B9" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-    </row>
-    <row r="10" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B10" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-    </row>
-    <row r="11" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B11" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-    </row>
-    <row r="12" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B12" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-    </row>
-    <row r="13" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B13" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-    </row>
-    <row r="14" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B14" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-    </row>
-    <row r="15" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B15" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-    </row>
-    <row r="16" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B16" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-    </row>
-    <row r="17" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B17" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-    </row>
-    <row r="18" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B18" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-    </row>
-    <row r="19" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B19" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-    </row>
-    <row r="20" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B20" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-    </row>
-    <row r="21" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B21" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-    </row>
-    <row r="22" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B22" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-    </row>
-    <row r="23" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B23" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-    </row>
-    <row r="24" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B24" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>